<commit_message>
Learn't about charts like boxplot,waterfall
</commit_message>
<xml_diff>
--- a/excelhw/Advanced Excel - Stu.xlsx
+++ b/excelhw/Advanced Excel - Stu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omsup\Documents\Advanced Excel\excelhw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF3E8D0-82B6-4942-992A-5CE27D628CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A1BF22-7F30-452D-8B9B-9D75B7BD044F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulas" sheetId="19" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6319" uniqueCount="3552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6331" uniqueCount="3554">
   <si>
     <t>State</t>
   </si>
@@ -10769,12 +10769,18 @@
   <si>
     <t>ki sab me changes hojaye</t>
   </si>
+  <si>
+    <t>doubt</t>
+  </si>
+  <si>
+    <t>All Division Summary</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
+  <numFmts count="13">
     <numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -10786,6 +10792,8 @@
     <numFmt numFmtId="169" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
+    <numFmt numFmtId="175" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="176" formatCode="dd\-mm\-yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="37" x14ac:knownFonts="1">
     <font>
@@ -11480,7 +11488,7 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11759,11 +11767,21 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="14" fillId="22" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="22"/>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="22" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="6" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="12" borderId="19" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -11783,21 +11801,6 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="6" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="18" borderId="7" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -11813,7 +11816,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="17" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="22"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="14" fillId="22" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="17" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="20% - Accent2" xfId="12" builtinId="34"/>
@@ -11840,7 +11855,221 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
     <cellStyle name="Title" xfId="3" builtinId="15"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="26">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -11852,6 +12081,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF3300"/>
+      <color rgb="FF669900"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FF0EBE27"/>
+      <color rgb="FF7EE888"/>
       <color rgb="FF99FFCC"/>
       <color rgb="FFFF6699"/>
     </mruColors>
@@ -13537,14 +13771,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>50800</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>424180</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>234950</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>6350</xdr:colOff>
       <xdr:row>13</xdr:row>
       <xdr:rowOff>139700</xdr:rowOff>
     </xdr:to>
@@ -13576,8 +13810,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="4495800" y="768350"/>
-          <a:ext cx="3232150" cy="1447800"/>
+          <a:off x="6611620" y="797560"/>
+          <a:ext cx="3194050" cy="1521460"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16514,15 +16748,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="117" t="s">
+      <c r="A1" s="121" t="s">
         <v>3463</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="1:7" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.45">
@@ -16535,11 +16769,11 @@
       <c r="C3" s="76" t="s">
         <v>3459</v>
       </c>
-      <c r="E3" s="112" t="s">
+      <c r="E3" s="116" t="s">
         <v>3461</v>
       </c>
-      <c r="F3" s="113"/>
-      <c r="G3" s="114"/>
+      <c r="F3" s="117"/>
+      <c r="G3" s="118"/>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="73" t="s">
@@ -16669,10 +16903,10 @@
     </row>
     <row r="11" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:7" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="115" t="s">
+      <c r="A12" s="119" t="s">
         <v>3452</v>
       </c>
-      <c r="B12" s="116"/>
+      <c r="B12" s="120"/>
       <c r="C12" s="69" t="s">
         <v>3451</v>
       </c>
@@ -16711,21 +16945,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="124" t="s">
+      <c r="A2" s="123" t="s">
         <v>3477</v>
       </c>
-      <c r="B2" s="125"/>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
+      <c r="B2" s="124"/>
+      <c r="C2" s="124"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="124"/>
+      <c r="F2" s="124"/>
+      <c r="G2" s="124"/>
     </row>
     <row r="4" spans="1:7" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="123" t="s">
+      <c r="A4" s="122" t="s">
         <v>3476</v>
       </c>
-      <c r="B4" s="123"/>
+      <c r="B4" s="122"/>
       <c r="E4" s="77" t="s">
         <v>3547</v>
       </c>
@@ -16766,15 +17000,15 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="123" t="s">
+      <c r="A10" s="122" t="s">
         <v>3474</v>
       </c>
-      <c r="B10" s="123"/>
-      <c r="C10" s="123"/>
-      <c r="D10" s="123"/>
-      <c r="E10" s="123"/>
-      <c r="F10" s="123"/>
-      <c r="G10" s="123"/>
+      <c r="B10" s="122"/>
+      <c r="C10" s="122"/>
+      <c r="D10" s="122"/>
+      <c r="E10" s="122"/>
+      <c r="F10" s="122"/>
+      <c r="G10" s="122"/>
     </row>
     <row r="11" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A11" s="78" t="s">
@@ -17176,7 +17410,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:D18">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="25" priority="1">
       <formula>AND($A2=$G$2,A$1=$G$3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17185,7 +17419,7 @@
       <formula1>$A$2:$A$18</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3" xr:uid="{C0192E8E-900D-4721-8825-1F06033C450E}">
-      <formula1>$B$2:$B$18</formula1>
+      <formula1>$B$1:$D$1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18231,7 +18465,7 @@
       <c r="L2">
         <v>62031</v>
       </c>
-      <c r="O2" s="128" t="s">
+      <c r="O2" s="110" t="s">
         <v>3301</v>
       </c>
       <c r="P2" s="45" t="str">
@@ -55704,7 +55938,7 @@
   <sheetPr>
     <tabColor theme="9" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
@@ -55715,650 +55949,746 @@
     <col min="7" max="7" width="16.44140625" style="98" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3522</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3521</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3520</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3519</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>3518</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="127">
         <v>41640</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="8">
         <v>1099</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="8">
         <v>275</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="8">
         <v>643</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="8">
         <f>B2-D2</f>
         <v>456</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="128">
         <f t="shared" ref="G2:G25" si="0">E2/B2</f>
         <v>0.41492265696087355</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="127">
         <v>41671</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="8">
         <v>1204</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="8">
         <f t="shared" ref="C3:C25" si="1">B3-B2</f>
         <v>105</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="8">
         <v>720</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="8">
         <v>211</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="128">
         <f t="shared" si="0"/>
         <v>0.17524916943521596</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="127">
         <v>41699</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="8">
         <v>1944</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="8">
         <f t="shared" si="1"/>
         <v>740</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="8">
         <v>964</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="8">
         <f t="shared" ref="E4:E19" si="2">B4-D4</f>
         <v>980</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="128">
         <f t="shared" si="0"/>
         <v>0.50411522633744854</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="127">
         <v>41730</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="8">
         <v>1743</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="8">
         <f t="shared" si="1"/>
         <v>-201</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="8">
         <v>830</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="8">
         <f t="shared" si="2"/>
         <v>913</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="128">
         <f t="shared" si="0"/>
         <v>0.52380952380952384</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" s="127">
         <v>41760</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="8">
         <v>1609</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="8">
         <f t="shared" si="1"/>
         <v>-134</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="8">
         <v>910</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="8">
         <f t="shared" si="2"/>
         <v>699</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="128">
         <f t="shared" si="0"/>
         <v>0.43443132380360472</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A7" s="127">
         <v>41791</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="8">
         <v>1494</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="8">
         <f t="shared" si="1"/>
         <v>-115</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="8">
         <v>909</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="8">
         <f t="shared" si="2"/>
         <v>585</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="128">
         <f t="shared" si="0"/>
         <v>0.39156626506024095</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A8" s="127">
         <v>41821</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="8">
         <v>1959</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="8">
         <f t="shared" si="1"/>
         <v>465</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="8">
         <v>830</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="8">
         <f t="shared" si="2"/>
         <v>1129</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="128">
         <f t="shared" si="0"/>
         <v>0.57631444614599281</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="127">
         <v>41852</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="8">
         <v>1868</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="8">
         <f t="shared" si="1"/>
         <v>-91</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="8">
         <v>906</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="8">
         <f t="shared" si="2"/>
         <v>962</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="128">
         <f t="shared" si="0"/>
         <v>0.51498929336188437</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A10" s="127">
         <v>41883</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="8">
         <v>1162</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="8">
         <f t="shared" si="1"/>
         <v>-706</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="8">
         <v>606</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="8">
         <f t="shared" si="2"/>
         <v>556</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="128">
         <f t="shared" si="0"/>
         <v>0.47848537005163511</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" s="127">
         <v>41913</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="8">
         <v>1424</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="8">
         <f t="shared" si="1"/>
         <v>262</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="8">
         <v>943</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="8">
         <f t="shared" si="2"/>
         <v>481</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="128">
         <f t="shared" si="0"/>
         <v>0.3377808988764045</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="127">
         <v>41944</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="8">
         <v>1232</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="8">
         <f t="shared" si="1"/>
         <v>-192</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="8">
         <v>801</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="8">
         <f t="shared" si="2"/>
         <v>431</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="128">
         <f t="shared" si="0"/>
         <v>0.34983766233766234</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="127">
         <v>41974</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="8">
         <v>1738</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="8">
         <f t="shared" si="1"/>
         <v>506</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="8">
         <v>786</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="8">
         <f t="shared" si="2"/>
         <v>952</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="128">
         <f t="shared" si="0"/>
         <v>0.54775604142692746</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="127">
         <v>42005</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="8">
         <v>1435</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="8">
         <f t="shared" si="1"/>
         <v>-303</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="8">
         <v>575</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="8">
         <f t="shared" si="2"/>
         <v>860</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="128">
         <f t="shared" si="0"/>
         <v>0.5993031358885017</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="127">
         <v>42036</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="8">
         <v>1865</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="8">
         <f t="shared" si="1"/>
         <v>430</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="8">
         <v>754</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="8">
         <f t="shared" si="2"/>
         <v>1111</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="128">
         <f t="shared" si="0"/>
         <v>0.59571045576407511</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16">
+      <c r="R15" t="s">
+        <v>3552</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="127">
         <v>42064</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="8">
         <v>1234</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="8">
         <f t="shared" si="1"/>
         <v>-631</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="8">
         <v>599</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="8">
         <f t="shared" si="2"/>
         <v>635</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="128">
         <f t="shared" si="0"/>
         <v>0.51458670988654787</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17" s="127">
         <v>42095</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="8">
         <v>1577</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="8">
         <f t="shared" si="1"/>
         <v>343</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="8">
         <v>940</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="8">
         <f t="shared" si="2"/>
         <v>637</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="128">
         <f t="shared" si="0"/>
         <v>0.40393151553582751</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18">
+      <c r="R17" t="s">
+        <v>3552</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="127">
         <v>42125</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="8">
         <v>1983</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="8">
         <f t="shared" si="1"/>
         <v>406</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="8">
         <v>954</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="8">
         <f t="shared" si="2"/>
         <v>1029</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="128">
         <f t="shared" si="0"/>
         <v>0.51891074130105896</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="127">
         <v>42156</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="8">
         <v>1356</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="8">
         <f t="shared" si="1"/>
         <v>-627</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="8">
         <v>577</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="8">
         <f t="shared" si="2"/>
         <v>779</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="128">
         <f t="shared" si="0"/>
         <v>0.57448377581120946</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="127">
         <v>42186</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="8">
         <v>1874</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="8">
         <f t="shared" si="1"/>
         <v>518</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="8">
         <v>865</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="8">
         <v>883</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="128">
         <f t="shared" si="0"/>
         <v>0.47118463180362863</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21" s="127">
         <v>42217</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="8">
         <v>1479</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="8">
         <f t="shared" si="1"/>
         <v>-395</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="8">
         <v>588</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="8">
         <f>B21-D21</f>
         <v>891</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="128">
         <f t="shared" si="0"/>
         <v>0.60243407707910746</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" s="127">
         <v>42248</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="8">
         <v>1943</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="8">
         <f t="shared" si="1"/>
         <v>464</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="8">
         <v>785</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="8">
         <v>712</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="128">
         <f t="shared" si="0"/>
         <v>0.36644364384971695</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" s="127">
         <v>42278</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="8">
         <v>1444</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="8">
         <f t="shared" si="1"/>
         <v>-499</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="8">
         <v>657</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="8">
         <f>B23-D23</f>
         <v>787</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="128">
         <f t="shared" si="0"/>
         <v>0.54501385041551242</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" s="127">
         <v>42309</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="8">
         <v>1493</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="8">
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="8">
         <v>880</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="8">
         <f>B24-D24</f>
         <v>613</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="128">
         <f t="shared" si="0"/>
         <v>0.4105827193569993</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" s="127">
         <v>42339</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="8">
         <v>1738</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="8">
         <f t="shared" si="1"/>
         <v>245</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="8">
         <v>580</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="8">
         <f>B25-D25</f>
         <v>1158</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="128">
         <f t="shared" si="0"/>
         <v>0.66628308400460301</v>
       </c>
+      <c r="O25" t="b">
+        <f>AND(G2&lt;40%)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O26" t="b">
+        <f t="shared" ref="O26:O35" si="3">AND(G3&lt;40%)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O27" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O28" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O29" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O30" t="b">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O31" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="O32" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="15:15" x14ac:dyDescent="0.3">
+      <c r="O33" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="15:15" x14ac:dyDescent="0.3">
+      <c r="O34" t="b">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="15:15" x14ac:dyDescent="0.3">
+      <c r="O35" t="b">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="G2:G25">
+    <cfRule type="cellIs" dxfId="9" priority="6" operator="lessThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="greaterThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="greaterThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
+      <formula>0.421</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:C25">
+    <cfRule type="iconSet" priority="1">
+      <iconSet iconSet="3Arrows">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="num" val="200"/>
+        <cfvo type="num" val="200"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -56378,7 +56708,7 @@
     <col min="3" max="3" width="19" style="2" customWidth="1"/>
     <col min="4" max="4" width="12.5546875" customWidth="1"/>
     <col min="5" max="5" width="11.77734375" customWidth="1"/>
-    <col min="6" max="6" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.21875" customWidth="1"/>
     <col min="8" max="8" width="20.21875" customWidth="1"/>
     <col min="9" max="9" width="15.5546875" customWidth="1"/>
@@ -56388,17 +56718,25 @@
       <c r="B2" s="109" t="s">
         <v>3546</v>
       </c>
-      <c r="C2" s="110"/>
+      <c r="C2" s="129">
+        <f ca="1">TODAY()</f>
+        <v>46225</v>
+      </c>
     </row>
     <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="109" t="s">
         <v>3545</v>
       </c>
-      <c r="C3" s="111"/>
+      <c r="C3" s="130">
+        <f ca="1">NOW()</f>
+        <v>46225.648052199074</v>
+      </c>
       <c r="E3" s="109" t="s">
         <v>3544</v>
       </c>
-      <c r="F3" s="110"/>
+      <c r="F3" s="129">
+        <v>46543</v>
+      </c>
     </row>
     <row r="4" spans="2:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="109"/>
@@ -56408,17 +56746,26 @@
       <c r="B5" s="9" t="s">
         <v>3543</v>
       </c>
-      <c r="C5" s="108"/>
+      <c r="C5" s="108">
+        <f ca="1">YEAR(TODAY())</f>
+        <v>2026</v>
+      </c>
       <c r="E5" s="9" t="s">
         <v>3542</v>
       </c>
-      <c r="F5" s="108"/>
+      <c r="F5" s="108">
+        <f ca="1">_xlfn.DAYS(F3,C2)</f>
+        <v>318</v>
+      </c>
     </row>
     <row r="6" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="9" t="s">
         <v>3541</v>
       </c>
-      <c r="C6" s="106"/>
+      <c r="C6" s="106">
+        <f ca="1">MONTH(TODAY())</f>
+        <v>7</v>
+      </c>
       <c r="E6" s="9" t="s">
         <v>3540</v>
       </c>
@@ -56428,7 +56775,10 @@
       <c r="B7" s="9" t="s">
         <v>3539</v>
       </c>
-      <c r="C7" s="106"/>
+      <c r="C7" s="106">
+        <f ca="1">DAY(TODAY())</f>
+        <v>22</v>
+      </c>
       <c r="E7" s="9" t="s">
         <v>3538</v>
       </c>
@@ -56439,13 +56789,19 @@
       <c r="B8" s="9" t="s">
         <v>3537</v>
       </c>
-      <c r="C8" s="106"/>
+      <c r="C8" s="106">
+        <f ca="1">HOUR(NOW())</f>
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="9" t="s">
         <v>3536</v>
       </c>
-      <c r="C9" s="106"/>
+      <c r="C9" s="106">
+        <f ca="1">MINUTE(NOW())</f>
+        <v>33</v>
+      </c>
       <c r="E9" s="9" t="s">
         <v>3535</v>
       </c>
@@ -56455,7 +56811,10 @@
       <c r="B10" s="9" t="s">
         <v>3534</v>
       </c>
-      <c r="C10" s="105"/>
+      <c r="C10" s="105">
+        <f ca="1">SECOND(NOW())</f>
+        <v>12</v>
+      </c>
       <c r="E10" s="9" t="s">
         <v>3533</v>
       </c>
@@ -56575,11 +56934,11 @@
       <c r="C9" s="53"/>
     </row>
     <row r="12" spans="1:3" ht="21" x14ac:dyDescent="0.4">
-      <c r="A12" s="126" t="s">
+      <c r="A12" s="125" t="s">
         <v>3328</v>
       </c>
-      <c r="B12" s="126"/>
-      <c r="C12" s="126"/>
+      <c r="B12" s="125"/>
+      <c r="C12" s="125"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="52" t="s">
@@ -56627,13 +56986,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="126" t="s">
         <v>3513</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57216,13 +57575,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="126" t="s">
         <v>3515</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57355,13 +57714,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="126" t="s">
         <v>3514</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57494,18 +57853,112 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="127"/>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
+      <c r="A1" s="126" t="s">
+        <v>3553</v>
+      </c>
+      <c r="B1" s="126"/>
+      <c r="C1" s="126"/>
+      <c r="D1" s="126"/>
+      <c r="E1" s="126"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="93" t="s">
+        <v>3511</v>
+      </c>
+      <c r="C2" s="93" t="s">
+        <v>3510</v>
+      </c>
+      <c r="D2" s="93" t="s">
+        <v>3509</v>
+      </c>
+      <c r="E2" s="93" t="s">
+        <v>3508</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="97"/>
-      <c r="B3" s="96"/>
-      <c r="C3" s="96"/>
-      <c r="D3" s="96"/>
-      <c r="E3" s="96"/>
+      <c r="A3" s="97" t="s">
+        <v>3487</v>
+      </c>
+      <c r="B3" s="96">
+        <v>800</v>
+      </c>
+      <c r="C3" s="96">
+        <v>2200</v>
+      </c>
+      <c r="D3" s="96">
+        <v>2500</v>
+      </c>
+      <c r="E3" s="96">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="93" t="s">
+        <v>3507</v>
+      </c>
+      <c r="B4" s="93">
+        <v>900</v>
+      </c>
+      <c r="C4" s="93">
+        <v>800</v>
+      </c>
+      <c r="D4" s="93">
+        <v>2500</v>
+      </c>
+      <c r="E4" s="93">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="93" t="s">
+        <v>3489</v>
+      </c>
+      <c r="B5" s="93">
+        <v>700</v>
+      </c>
+      <c r="C5" s="93">
+        <v>1300</v>
+      </c>
+      <c r="D5" s="93">
+        <v>2400</v>
+      </c>
+      <c r="E5" s="93">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="93" t="s">
+        <v>3506</v>
+      </c>
+      <c r="B6" s="93">
+        <v>600</v>
+      </c>
+      <c r="C6" s="93">
+        <v>900</v>
+      </c>
+      <c r="D6" s="93">
+        <v>1100</v>
+      </c>
+      <c r="E6" s="93">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="93" t="s">
+        <v>3505</v>
+      </c>
+      <c r="B7" s="131">
+        <v>3000</v>
+      </c>
+      <c r="C7" s="131">
+        <v>5200</v>
+      </c>
+      <c r="D7" s="131">
+        <v>8500</v>
+      </c>
+      <c r="E7" s="131">
+        <v>3400</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="95"/>
@@ -57515,7 +57968,7 @@
       <c r="E9" s="94"/>
     </row>
   </sheetData>
-  <dataConsolidate topLabels="1">
+  <dataConsolidate leftLabels="1" topLabels="1">
     <dataRefs count="3">
       <dataRef ref="A3:E9" sheet="Connecticut"/>
       <dataRef ref="A3:E9" sheet="Maine"/>
@@ -57882,14 +58335,14 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="111" t="s">
         <v>3504</v>
       </c>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="120"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="113"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="92" t="s">
@@ -69191,20 +69644,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="114" t="s">
         <v>3450</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
+      <c r="B1" s="114"/>
+      <c r="C1" s="114"/>
+      <c r="D1" s="114"/>
+      <c r="E1" s="114"/>
     </row>
     <row r="2" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="121"/>
-      <c r="B2" s="121"/>
-      <c r="C2" s="121"/>
-      <c r="D2" s="121"/>
-      <c r="E2" s="121"/>
+      <c r="A2" s="114"/>
+      <c r="B2" s="114"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="114"/>
+      <c r="E2" s="114"/>
     </row>
     <row r="3" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A3" s="64" t="s">
@@ -69245,28 +69698,28 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="122" t="s">
+      <c r="A7" s="115" t="s">
         <v>3449</v>
       </c>
-      <c r="B7" s="122"/>
-      <c r="C7" s="122"/>
-      <c r="D7" s="122"/>
-      <c r="E7" s="122"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="122"/>
-      <c r="H7" s="122"/>
-      <c r="I7" s="122"/>
+      <c r="B7" s="115"/>
+      <c r="C7" s="115"/>
+      <c r="D7" s="115"/>
+      <c r="E7" s="115"/>
+      <c r="F7" s="115"/>
+      <c r="G7" s="115"/>
+      <c r="H7" s="115"/>
+      <c r="I7" s="115"/>
     </row>
     <row r="8" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="121"/>
-      <c r="B8" s="121"/>
-      <c r="C8" s="121"/>
-      <c r="D8" s="121"/>
-      <c r="E8" s="121"/>
-      <c r="F8" s="121"/>
-      <c r="G8" s="121"/>
-      <c r="H8" s="121"/>
-      <c r="I8" s="121"/>
+      <c r="A8" s="114"/>
+      <c r="B8" s="114"/>
+      <c r="C8" s="114"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="114"/>
+      <c r="F8" s="114"/>
+      <c r="G8" s="114"/>
+      <c r="H8" s="114"/>
+      <c r="I8" s="114"/>
     </row>
     <row r="9" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A9" s="64" t="s">

</xml_diff>

<commit_message>
Learn't Date and Time Functions
</commit_message>
<xml_diff>
--- a/excelhw/Advanced Excel - Stu.xlsx
+++ b/excelhw/Advanced Excel - Stu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omsup\Documents\Advanced Excel\excelhw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A1BF22-7F30-452D-8B9B-9D75B7BD044F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF271A4-49FE-462B-98AB-02D7CE380BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulas" sheetId="19" r:id="rId1"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6331" uniqueCount="3554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6334" uniqueCount="3558">
   <si>
     <t>State</t>
   </si>
@@ -10775,6 +10775,18 @@
   <si>
     <t>All Division Summary</t>
   </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>sumifs</t>
+  </si>
+  <si>
+    <t>sumif</t>
+  </si>
+  <si>
+    <t>averageif</t>
+  </si>
 </sst>
 </file>
 
@@ -10792,8 +10804,8 @@
     <numFmt numFmtId="169" formatCode="dd\-mmm\-yy"/>
     <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="171" formatCode="0.0%"/>
-    <numFmt numFmtId="175" formatCode="dd\-mm\-yyyy"/>
-    <numFmt numFmtId="176" formatCode="dd\-mm\-yyyy\ hh:mm"/>
+    <numFmt numFmtId="172" formatCode="dd\-mm\-yyyy"/>
+    <numFmt numFmtId="173" formatCode="dd\-mm\-yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="37" x14ac:knownFonts="1">
     <font>
@@ -11768,21 +11780,19 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="22"/>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="172" fontId="14" fillId="22" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="6" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="173" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="17" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="26" fillId="12" borderId="19" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -11801,6 +11811,21 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="19" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="17" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="6" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="18" borderId="7" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -11816,19 +11841,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="17" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="14" fillId="22" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="14" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="17" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="23">
     <cellStyle name="20% - Accent2" xfId="12" builtinId="34"/>
@@ -11855,181 +11867,7 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
     <cellStyle name="Title" xfId="3" builtinId="15"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF3300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0EBE27"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF3300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0EBE27"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF3300"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0EBE27"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0EBE27"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0EBE27"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -12051,22 +11889,23 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF0EBE27"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
         </patternFill>
       </fill>
     </dxf>
@@ -15630,16 +15469,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>152400</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>222250</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>496570</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>120650</xdr:rowOff>
+      <xdr:rowOff>181610</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -15669,8 +15508,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="5664200" y="2451100"/>
-          <a:ext cx="3568700" cy="1993900"/>
+          <a:off x="7741920" y="2515870"/>
+          <a:ext cx="3506470" cy="1986280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16787,7 +16626,7 @@
         <v>124</v>
       </c>
       <c r="F4" s="74" t="s">
-        <v>3459</v>
+        <v>3554</v>
       </c>
       <c r="G4" s="74" t="s">
         <v>3451</v>
@@ -16908,7 +16747,7 @@
       </c>
       <c r="B12" s="120"/>
       <c r="C12" s="69" t="s">
-        <v>3451</v>
+        <v>3554</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
@@ -16945,21 +16784,21 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="123" t="s">
+      <c r="A2" s="128" t="s">
         <v>3477</v>
       </c>
-      <c r="B2" s="124"/>
-      <c r="C2" s="124"/>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
+      <c r="B2" s="129"/>
+      <c r="C2" s="129"/>
+      <c r="D2" s="129"/>
+      <c r="E2" s="129"/>
+      <c r="F2" s="129"/>
+      <c r="G2" s="129"/>
     </row>
     <row r="4" spans="1:7" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="122" t="s">
+      <c r="A4" s="127" t="s">
         <v>3476</v>
       </c>
-      <c r="B4" s="122"/>
+      <c r="B4" s="127"/>
       <c r="E4" s="77" t="s">
         <v>3547</v>
       </c>
@@ -17000,15 +16839,15 @@
       </c>
     </row>
     <row r="10" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="122" t="s">
+      <c r="A10" s="127" t="s">
         <v>3474</v>
       </c>
-      <c r="B10" s="122"/>
-      <c r="C10" s="122"/>
-      <c r="D10" s="122"/>
-      <c r="E10" s="122"/>
-      <c r="F10" s="122"/>
-      <c r="G10" s="122"/>
+      <c r="B10" s="127"/>
+      <c r="C10" s="127"/>
+      <c r="D10" s="127"/>
+      <c r="E10" s="127"/>
+      <c r="F10" s="127"/>
+      <c r="G10" s="127"/>
     </row>
     <row r="11" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A11" s="78" t="s">
@@ -17410,7 +17249,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:D18">
-    <cfRule type="expression" dxfId="25" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>AND($A2=$G$2,A$1=$G$3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -55973,7 +55812,7 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A2" s="127">
+      <c r="A2" s="111">
         <v>41640</v>
       </c>
       <c r="B2" s="8">
@@ -55992,13 +55831,13 @@
       <c r="F2" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G2" s="128">
+      <c r="G2" s="112">
         <f t="shared" ref="G2:G25" si="0">E2/B2</f>
         <v>0.41492265696087355</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A3" s="127">
+      <c r="A3" s="111">
         <v>41671</v>
       </c>
       <c r="B3" s="8">
@@ -56017,13 +55856,13 @@
       <c r="F3" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G3" s="128">
+      <c r="G3" s="112">
         <f t="shared" si="0"/>
         <v>0.17524916943521596</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A4" s="127">
+      <c r="A4" s="111">
         <v>41699</v>
       </c>
       <c r="B4" s="8">
@@ -56043,13 +55882,13 @@
       <c r="F4" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G4" s="128">
+      <c r="G4" s="112">
         <f t="shared" si="0"/>
         <v>0.50411522633744854</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A5" s="127">
+      <c r="A5" s="111">
         <v>41730</v>
       </c>
       <c r="B5" s="8">
@@ -56069,13 +55908,13 @@
       <c r="F5" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G5" s="128">
+      <c r="G5" s="112">
         <f t="shared" si="0"/>
         <v>0.52380952380952384</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A6" s="127">
+      <c r="A6" s="111">
         <v>41760</v>
       </c>
       <c r="B6" s="8">
@@ -56095,13 +55934,13 @@
       <c r="F6" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G6" s="128">
+      <c r="G6" s="112">
         <f t="shared" si="0"/>
         <v>0.43443132380360472</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A7" s="127">
+      <c r="A7" s="111">
         <v>41791</v>
       </c>
       <c r="B7" s="8">
@@ -56121,13 +55960,13 @@
       <c r="F7" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="128">
+      <c r="G7" s="112">
         <f t="shared" si="0"/>
         <v>0.39156626506024095</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A8" s="127">
+      <c r="A8" s="111">
         <v>41821</v>
       </c>
       <c r="B8" s="8">
@@ -56147,13 +55986,13 @@
       <c r="F8" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G8" s="128">
+      <c r="G8" s="112">
         <f t="shared" si="0"/>
         <v>0.57631444614599281</v>
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="127">
+      <c r="A9" s="111">
         <v>41852</v>
       </c>
       <c r="B9" s="8">
@@ -56173,13 +56012,13 @@
       <c r="F9" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G9" s="128">
+      <c r="G9" s="112">
         <f t="shared" si="0"/>
         <v>0.51498929336188437</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A10" s="127">
+      <c r="A10" s="111">
         <v>41883</v>
       </c>
       <c r="B10" s="8">
@@ -56199,13 +56038,13 @@
       <c r="F10" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G10" s="128">
+      <c r="G10" s="112">
         <f t="shared" si="0"/>
         <v>0.47848537005163511</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A11" s="127">
+      <c r="A11" s="111">
         <v>41913</v>
       </c>
       <c r="B11" s="8">
@@ -56225,13 +56064,13 @@
       <c r="F11" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G11" s="128">
+      <c r="G11" s="112">
         <f t="shared" si="0"/>
         <v>0.3377808988764045</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A12" s="127">
+      <c r="A12" s="111">
         <v>41944</v>
       </c>
       <c r="B12" s="8">
@@ -56251,13 +56090,13 @@
       <c r="F12" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G12" s="128">
+      <c r="G12" s="112">
         <f t="shared" si="0"/>
         <v>0.34983766233766234</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A13" s="127">
+      <c r="A13" s="111">
         <v>41974</v>
       </c>
       <c r="B13" s="8">
@@ -56277,13 +56116,13 @@
       <c r="F13" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G13" s="128">
+      <c r="G13" s="112">
         <f t="shared" si="0"/>
         <v>0.54775604142692746</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A14" s="127">
+      <c r="A14" s="111">
         <v>42005</v>
       </c>
       <c r="B14" s="8">
@@ -56303,13 +56142,13 @@
       <c r="F14" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G14" s="128">
+      <c r="G14" s="112">
         <f t="shared" si="0"/>
         <v>0.5993031358885017</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A15" s="127">
+      <c r="A15" s="111">
         <v>42036</v>
       </c>
       <c r="B15" s="8">
@@ -56329,7 +56168,7 @@
       <c r="F15" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G15" s="128">
+      <c r="G15" s="112">
         <f t="shared" si="0"/>
         <v>0.59571045576407511</v>
       </c>
@@ -56338,7 +56177,7 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A16" s="127">
+      <c r="A16" s="111">
         <v>42064</v>
       </c>
       <c r="B16" s="8">
@@ -56358,13 +56197,13 @@
       <c r="F16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G16" s="128">
+      <c r="G16" s="112">
         <f t="shared" si="0"/>
         <v>0.51458670988654787</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A17" s="127">
+      <c r="A17" s="111">
         <v>42095</v>
       </c>
       <c r="B17" s="8">
@@ -56384,7 +56223,7 @@
       <c r="F17" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G17" s="128">
+      <c r="G17" s="112">
         <f t="shared" si="0"/>
         <v>0.40393151553582751</v>
       </c>
@@ -56393,7 +56232,7 @@
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A18" s="127">
+      <c r="A18" s="111">
         <v>42125</v>
       </c>
       <c r="B18" s="8">
@@ -56413,13 +56252,13 @@
       <c r="F18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G18" s="128">
+      <c r="G18" s="112">
         <f t="shared" si="0"/>
         <v>0.51891074130105896</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A19" s="127">
+      <c r="A19" s="111">
         <v>42156</v>
       </c>
       <c r="B19" s="8">
@@ -56439,13 +56278,13 @@
       <c r="F19" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G19" s="128">
+      <c r="G19" s="112">
         <f t="shared" si="0"/>
         <v>0.57448377581120946</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A20" s="127">
+      <c r="A20" s="111">
         <v>42186</v>
       </c>
       <c r="B20" s="8">
@@ -56464,13 +56303,13 @@
       <c r="F20" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G20" s="128">
+      <c r="G20" s="112">
         <f t="shared" si="0"/>
         <v>0.47118463180362863</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A21" s="127">
+      <c r="A21" s="111">
         <v>42217</v>
       </c>
       <c r="B21" s="8">
@@ -56490,13 +56329,13 @@
       <c r="F21" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G21" s="128">
+      <c r="G21" s="112">
         <f t="shared" si="0"/>
         <v>0.60243407707910746</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A22" s="127">
+      <c r="A22" s="111">
         <v>42248</v>
       </c>
       <c r="B22" s="8">
@@ -56515,13 +56354,13 @@
       <c r="F22" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G22" s="128">
+      <c r="G22" s="112">
         <f t="shared" si="0"/>
         <v>0.36644364384971695</v>
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A23" s="127">
+      <c r="A23" s="111">
         <v>42278</v>
       </c>
       <c r="B23" s="8">
@@ -56541,13 +56380,13 @@
       <c r="F23" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="G23" s="128">
+      <c r="G23" s="112">
         <f t="shared" si="0"/>
         <v>0.54501385041551242</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A24" s="127">
+      <c r="A24" s="111">
         <v>42309</v>
       </c>
       <c r="B24" s="8">
@@ -56567,13 +56406,13 @@
       <c r="F24" s="2" t="s">
         <v>3517</v>
       </c>
-      <c r="G24" s="128">
+      <c r="G24" s="112">
         <f t="shared" si="0"/>
         <v>0.4105827193569993</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A25" s="127">
+      <c r="A25" s="111">
         <v>42339</v>
       </c>
       <c r="B25" s="8">
@@ -56593,7 +56432,7 @@
       <c r="F25" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="G25" s="128">
+      <c r="G25" s="112">
         <f t="shared" si="0"/>
         <v>0.66628308400460301</v>
       </c>
@@ -56663,23 +56502,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="G2:G25">
-    <cfRule type="cellIs" dxfId="9" priority="6" operator="lessThan">
-      <formula>0.421</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="greaterThan">
-      <formula>0.421</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="greaterThan">
-      <formula>0.421</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="lessThan">
-      <formula>0.421</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="lessThan">
-      <formula>0.421</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C2:C25">
     <cfRule type="iconSet" priority="1">
       <iconSet iconSet="3Arrows">
@@ -56687,6 +56509,23 @@
         <cfvo type="num" val="200"/>
         <cfvo type="num" val="200"/>
       </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G25">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="greaterThan">
+      <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="6" operator="lessThan">
+      <formula>0.421</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56718,23 +56557,23 @@
       <c r="B2" s="109" t="s">
         <v>3546</v>
       </c>
-      <c r="C2" s="129">
+      <c r="C2" s="113">
         <f ca="1">TODAY()</f>
-        <v>46225</v>
+        <v>46228</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="109" t="s">
         <v>3545</v>
       </c>
-      <c r="C3" s="130">
+      <c r="C3" s="114">
         <f ca="1">NOW()</f>
-        <v>46225.648052199074</v>
+        <v>46228.381456944444</v>
       </c>
       <c r="E3" s="109" t="s">
         <v>3544</v>
       </c>
-      <c r="F3" s="129">
+      <c r="F3" s="113">
         <v>46543</v>
       </c>
     </row>
@@ -56755,7 +56594,7 @@
       </c>
       <c r="F5" s="108">
         <f ca="1">_xlfn.DAYS(F3,C2)</f>
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -56777,7 +56616,7 @@
       </c>
       <c r="C7" s="106">
         <f ca="1">DAY(TODAY())</f>
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>3538</v>
@@ -56791,7 +56630,7 @@
       </c>
       <c r="C8" s="106">
         <f ca="1">HOUR(NOW())</f>
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -56800,7 +56639,7 @@
       </c>
       <c r="C9" s="106">
         <f ca="1">MINUTE(NOW())</f>
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>3535</v>
@@ -56813,7 +56652,7 @@
       </c>
       <c r="C10" s="105">
         <f ca="1">SECOND(NOW())</f>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>3533</v>
@@ -56934,11 +56773,11 @@
       <c r="C9" s="53"/>
     </row>
     <row r="12" spans="1:3" ht="21" x14ac:dyDescent="0.4">
-      <c r="A12" s="125" t="s">
+      <c r="A12" s="130" t="s">
         <v>3328</v>
       </c>
-      <c r="B12" s="125"/>
-      <c r="C12" s="125"/>
+      <c r="B12" s="130"/>
+      <c r="C12" s="130"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="52" t="s">
@@ -56986,13 +56825,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="131" t="s">
         <v>3513</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57575,13 +57414,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="131" t="s">
         <v>3515</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57714,13 +57553,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="131" t="s">
         <v>3514</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="97" t="s">
@@ -57853,13 +57692,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="131" t="s">
         <v>3553</v>
       </c>
-      <c r="B1" s="126"/>
-      <c r="C1" s="126"/>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" s="93" t="s">
@@ -57947,16 +57786,16 @@
       <c r="A7" s="93" t="s">
         <v>3505</v>
       </c>
-      <c r="B7" s="131">
+      <c r="B7" s="115">
         <v>3000</v>
       </c>
-      <c r="C7" s="131">
+      <c r="C7" s="115">
         <v>5200</v>
       </c>
-      <c r="D7" s="131">
+      <c r="D7" s="115">
         <v>8500</v>
       </c>
-      <c r="E7" s="131">
+      <c r="E7" s="115">
         <v>3400</v>
       </c>
     </row>
@@ -57968,7 +57807,7 @@
       <c r="E9" s="94"/>
     </row>
   </sheetData>
-  <dataConsolidate leftLabels="1" topLabels="1">
+  <dataConsolidate topLabels="1">
     <dataRefs count="3">
       <dataRef ref="A3:E9" sheet="Connecticut"/>
       <dataRef ref="A3:E9" sheet="Maine"/>
@@ -58335,14 +58174,14 @@
   <sheetData>
     <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:12" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="122" t="s">
         <v>3504</v>
       </c>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="113"/>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="123"/>
+      <c r="F2" s="123"/>
+      <c r="G2" s="124"/>
     </row>
     <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="92" t="s">
@@ -58385,6 +58224,9 @@
         <f>SUM(D5:F5)</f>
         <v>2150</v>
       </c>
+      <c r="K5" s="49" t="s">
+        <v>3555</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="60"/>
@@ -58470,7 +58312,10 @@
       <c r="J8" s="85" t="s">
         <v>3487</v>
       </c>
-      <c r="K8" s="89"/>
+      <c r="K8" s="89">
+        <f>SUMIFS(G5:G62,B5:B62,I8,C5:C62,J8)</f>
+        <v>5875</v>
+      </c>
       <c r="L8" s="88"/>
     </row>
     <row r="9" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -58561,6 +58406,9 @@
         <f t="shared" si="0"/>
         <v>11300</v>
       </c>
+      <c r="K12" s="49" t="s">
+        <v>3556</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="60"/>
@@ -58614,7 +58462,10 @@
       <c r="I14" s="85" t="s">
         <v>3487</v>
       </c>
-      <c r="J14" s="84"/>
+      <c r="J14" s="84">
+        <f>SUMIF(C5:C62,I14,G5:G62)</f>
+        <v>17215</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="60"/>
@@ -58660,7 +58511,7 @@
         <v>36500</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="60"/>
       <c r="B17" s="87" t="s">
         <v>3497</v>
@@ -58681,8 +58532,11 @@
         <f t="shared" si="0"/>
         <v>37250</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" s="49" t="s">
+        <v>3557</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="60"/>
       <c r="B18" s="87" t="s">
         <v>3497</v>
@@ -58704,7 +58558,7 @@
         <v>75390</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="60"/>
       <c r="B19" s="83" t="s">
         <v>3494</v>
@@ -58732,7 +58586,7 @@
         <v>3495</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B20" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58755,9 +58609,12 @@
       <c r="I20" s="85" t="s">
         <v>3484</v>
       </c>
-      <c r="J20" s="84"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J20" s="84">
+        <f>AVERAGEIF(C5:C62,I20,G5:G62)</f>
+        <v>17790</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B21" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58778,7 +58635,7 @@
         <v>2710</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B22" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58799,7 +58656,7 @@
         <v>2780</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B23" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58820,7 +58677,7 @@
         <v>3750</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B24" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58841,7 +58698,7 @@
         <v>3805</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B25" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58862,7 +58719,7 @@
         <v>6650</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B26" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58883,7 +58740,7 @@
         <v>10710</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B27" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58904,7 +58761,7 @@
         <v>14300</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B28" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58925,7 +58782,7 @@
         <v>19755</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B29" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58946,7 +58803,7 @@
         <v>18060</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B30" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58967,7 +58824,7 @@
         <v>35740</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B31" s="83" t="s">
         <v>3494</v>
       </c>
@@ -58988,7 +58845,7 @@
         <v>41550</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B32" s="83" t="s">
         <v>3494</v>
       </c>
@@ -69644,20 +69501,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="114" t="s">
+      <c r="A1" s="125" t="s">
         <v>3450</v>
       </c>
-      <c r="B1" s="114"/>
-      <c r="C1" s="114"/>
-      <c r="D1" s="114"/>
-      <c r="E1" s="114"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
     </row>
     <row r="2" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="114"/>
-      <c r="B2" s="114"/>
-      <c r="C2" s="114"/>
-      <c r="D2" s="114"/>
-      <c r="E2" s="114"/>
+      <c r="A2" s="125"/>
+      <c r="B2" s="125"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
     </row>
     <row r="3" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A3" s="64" t="s">
@@ -69698,28 +69555,28 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="115" t="s">
+      <c r="A7" s="126" t="s">
         <v>3449</v>
       </c>
-      <c r="B7" s="115"/>
-      <c r="C7" s="115"/>
-      <c r="D7" s="115"/>
-      <c r="E7" s="115"/>
-      <c r="F7" s="115"/>
-      <c r="G7" s="115"/>
-      <c r="H7" s="115"/>
-      <c r="I7" s="115"/>
+      <c r="B7" s="126"/>
+      <c r="C7" s="126"/>
+      <c r="D7" s="126"/>
+      <c r="E7" s="126"/>
+      <c r="F7" s="126"/>
+      <c r="G7" s="126"/>
+      <c r="H7" s="126"/>
+      <c r="I7" s="126"/>
     </row>
     <row r="8" spans="1:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="114"/>
-      <c r="B8" s="114"/>
-      <c r="C8" s="114"/>
-      <c r="D8" s="114"/>
-      <c r="E8" s="114"/>
-      <c r="F8" s="114"/>
-      <c r="G8" s="114"/>
-      <c r="H8" s="114"/>
-      <c r="I8" s="114"/>
+      <c r="A8" s="125"/>
+      <c r="B8" s="125"/>
+      <c r="C8" s="125"/>
+      <c r="D8" s="125"/>
+      <c r="E8" s="125"/>
+      <c r="F8" s="125"/>
+      <c r="G8" s="125"/>
+      <c r="H8" s="125"/>
+      <c r="I8" s="125"/>
     </row>
     <row r="9" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A9" s="64" t="s">

</xml_diff>

<commit_message>
Solved Standard and Holiday Bonus assign using nested if
</commit_message>
<xml_diff>
--- a/excelhw/Advanced Excel - Stu.xlsx
+++ b/excelhw/Advanced Excel - Stu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omsup\Documents\Advanced Excel\excelhw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF271A4-49FE-462B-98AB-02D7CE380BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1491149D-80F4-42BB-9D90-700669C34448}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="645" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Formulas" sheetId="19" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6334" uniqueCount="3558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6370" uniqueCount="3572">
   <si>
     <t>State</t>
   </si>
@@ -10770,9 +10770,6 @@
     <t>ki sab me changes hojaye</t>
   </si>
   <si>
-    <t>doubt</t>
-  </si>
-  <si>
     <t>All Division Summary</t>
   </si>
   <si>
@@ -10786,6 +10783,51 @@
   </si>
   <si>
     <t>averageif</t>
+  </si>
+  <si>
+    <t>1000-1500</t>
+  </si>
+  <si>
+    <t>1500-2000</t>
+  </si>
+  <si>
+    <t>2000-2500</t>
+  </si>
+  <si>
+    <t>2500-3000</t>
+  </si>
+  <si>
+    <t>3000-3500</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>3500-4000</t>
+  </si>
+  <si>
+    <t>std</t>
+  </si>
+  <si>
+    <t>4000-4500</t>
+  </si>
+  <si>
+    <t>4500-5000</t>
+  </si>
+  <si>
+    <t>0-1000</t>
+  </si>
+  <si>
+    <t>range is not continuous ki ham koi decision pr aaye</t>
+  </si>
+  <si>
+    <t>holiday</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>kids</t>
   </si>
 </sst>
 </file>
@@ -11867,7 +11909,675 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
     <cellStyle name="Title" xfId="3" builtinId="15"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="88">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF3300"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0EBE27"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF3300"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -12825,16 +13535,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>200024</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>323591</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>70485</xdr:rowOff>
+      <xdr:rowOff>163160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>182879</xdr:colOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>306446</xdr:colOff>
       <xdr:row>20</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:rowOff>138395</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -12849,8 +13559,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4467224" y="254635"/>
-          <a:ext cx="5469255" cy="3474085"/>
+          <a:off x="11104861" y="348511"/>
+          <a:ext cx="5450720" cy="3496911"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14017,16 +14727,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1033780</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>68581</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>203200</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>99061</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>547370</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>158750</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14041,8 +14751,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4767580" y="1725931"/>
-          <a:ext cx="8594090" cy="2056129"/>
+          <a:off x="4919980" y="2110741"/>
+          <a:ext cx="8505190" cy="2042159"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16575,7 +17285,7 @@
   <sheetPr>
     <tabColor rgb="FF002060"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="17" style="49" customWidth="1"/>
@@ -16621,12 +17331,15 @@
       <c r="B4" s="72">
         <v>1200</v>
       </c>
-      <c r="C4" s="71"/>
+      <c r="C4" s="71">
+        <f>IF(B4&lt;1000,0,IF(B4&lt;1500,10,IF(B4&lt;2000,30,IF(B4&lt;2500,85,IF(B4&lt;3000,125,IF(B4&lt;3500,200,IF(B4&lt;5000,200)))))))</f>
+        <v>10</v>
+      </c>
       <c r="E4" s="75" t="s">
         <v>124</v>
       </c>
       <c r="F4" s="74" t="s">
-        <v>3554</v>
+        <v>3553</v>
       </c>
       <c r="G4" s="74" t="s">
         <v>3451</v>
@@ -16639,7 +17352,10 @@
       <c r="B5" s="72">
         <v>1300</v>
       </c>
-      <c r="C5" s="71"/>
+      <c r="C5" s="71">
+        <f t="shared" ref="C5:C10" si="0">IF(B5&lt;1000,0,IF(B5&lt;1500,10,IF(B5&lt;2000,30,IF(B5&lt;2500,85,IF(B5&lt;3000,125,IF(B5&lt;3500,200,IF(B5&lt;5000,200)))))))</f>
+        <v>10</v>
+      </c>
       <c r="E5" s="70">
         <v>0</v>
       </c>
@@ -16657,7 +17373,10 @@
       <c r="B6" s="72">
         <v>2500</v>
       </c>
-      <c r="C6" s="71"/>
+      <c r="C6" s="71">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
       <c r="E6" s="70">
         <v>1000</v>
       </c>
@@ -16675,7 +17394,10 @@
       <c r="B7" s="72">
         <v>850</v>
       </c>
-      <c r="C7" s="71"/>
+      <c r="C7" s="71">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="E7" s="70">
         <v>1500</v>
       </c>
@@ -16693,7 +17415,10 @@
       <c r="B8" s="72">
         <v>3250</v>
       </c>
-      <c r="C8" s="71"/>
+      <c r="C8" s="71">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
       <c r="E8" s="70">
         <v>2000</v>
       </c>
@@ -16711,7 +17436,10 @@
       <c r="B9" s="72">
         <v>1100</v>
       </c>
-      <c r="C9" s="71"/>
+      <c r="C9" s="71">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="E9" s="70">
         <v>2500</v>
       </c>
@@ -16729,7 +17457,10 @@
       <c r="B10" s="72">
         <v>4520</v>
       </c>
-      <c r="C10" s="71"/>
+      <c r="C10" s="71">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
       <c r="E10" s="70">
         <v>3000</v>
       </c>
@@ -16747,20 +17478,266 @@
       </c>
       <c r="B12" s="120"/>
       <c r="C12" s="69" t="s">
-        <v>3554</v>
+        <v>3553</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="E13" s="68"/>
-    </row>
+      <c r="E13" s="68" t="s">
+        <v>3564</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E14" s="49" t="s">
+        <v>3567</v>
+      </c>
+      <c r="F14" s="49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="49" t="s">
+        <v>3569</v>
+      </c>
+      <c r="E15" s="49" t="s">
+        <v>3557</v>
+      </c>
+      <c r="F15" s="49">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="49" t="s">
+        <v>3567</v>
+      </c>
+      <c r="B16" s="49">
+        <v>0</v>
+      </c>
+      <c r="E16" s="49" t="s">
+        <v>3558</v>
+      </c>
+      <c r="F16" s="49">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="49" t="s">
+        <v>3557</v>
+      </c>
+      <c r="B17" s="49">
+        <v>20</v>
+      </c>
+      <c r="E17" s="49" t="s">
+        <v>3559</v>
+      </c>
+      <c r="F17" s="49">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="49" t="s">
+        <v>3558</v>
+      </c>
+      <c r="B18" s="49">
+        <v>50</v>
+      </c>
+      <c r="E18" s="49" t="s">
+        <v>3560</v>
+      </c>
+      <c r="F18" s="49">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="49" t="s">
+        <v>3559</v>
+      </c>
+      <c r="B19" s="49">
+        <v>100</v>
+      </c>
+      <c r="E19" s="49" t="s">
+        <v>3561</v>
+      </c>
+      <c r="F19" s="49">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="49" t="s">
+        <v>3560</v>
+      </c>
+      <c r="B20" s="49">
+        <v>150</v>
+      </c>
+      <c r="E20" s="49" t="s">
+        <v>3563</v>
+      </c>
+      <c r="F20" s="49">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="49" t="s">
+        <v>3561</v>
+      </c>
+      <c r="B21" s="49">
+        <v>250</v>
+      </c>
+      <c r="E21" s="49" t="s">
+        <v>3565</v>
+      </c>
+      <c r="F21" s="49" t="s">
+        <v>3562</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="49" t="s">
+        <v>3563</v>
+      </c>
+      <c r="B22" s="49" t="s">
+        <v>3562</v>
+      </c>
+      <c r="E22" s="49" t="s">
+        <v>3566</v>
+      </c>
+      <c r="F22" s="49">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="49" t="s">
+        <v>3565</v>
+      </c>
+      <c r="B23" s="49" t="s">
+        <v>3562</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="49" t="s">
+        <v>3566</v>
+      </c>
+      <c r="B24" s="49">
+        <v>250</v>
+      </c>
+      <c r="E24" s="49" t="s">
+        <v>3568</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="27" spans="1:6" ht="20.399999999999999" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="76" t="s">
+        <v>3462</v>
+      </c>
+      <c r="B27" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="76" t="s">
+        <v>3459</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="73" t="s">
+        <v>3460</v>
+      </c>
+      <c r="B28" s="72">
+        <v>1200</v>
+      </c>
+      <c r="C28" s="71">
+        <f>IF(B28&lt;1000,0,IF(B28&lt;1500,20,IF(B28&lt;2000,50,IF(B28&lt;2500,100,IF(B28&lt;3000,150,IF(B28&lt;3500,250,IF(B28&lt;5000,250)))))))</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="73" t="s">
+        <v>3458</v>
+      </c>
+      <c r="B29" s="72">
+        <v>1300</v>
+      </c>
+      <c r="C29" s="71">
+        <f t="shared" ref="C29:C34" si="1">IF(B29&lt;1000,0,IF(B29&lt;1500,20,IF(B29&lt;2000,50,IF(B29&lt;2500,100,IF(B29&lt;3000,150,IF(B29&lt;3500,250,IF(B29&lt;5000,250)))))))</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="73" t="s">
+        <v>3457</v>
+      </c>
+      <c r="B30" s="72">
+        <v>2500</v>
+      </c>
+      <c r="C30" s="71">
+        <f t="shared" si="1"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="73" t="s">
+        <v>3456</v>
+      </c>
+      <c r="B31" s="72">
+        <v>850</v>
+      </c>
+      <c r="C31" s="71">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="73" t="s">
+        <v>3455</v>
+      </c>
+      <c r="B32" s="72">
+        <v>3250</v>
+      </c>
+      <c r="C32" s="71">
+        <f t="shared" si="1"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="73" t="s">
+        <v>3454</v>
+      </c>
+      <c r="B33" s="72">
+        <v>1100</v>
+      </c>
+      <c r="C33" s="71">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="73" t="s">
+        <v>3453</v>
+      </c>
+      <c r="B34" s="72">
+        <v>4520</v>
+      </c>
+      <c r="C34" s="71">
+        <f t="shared" si="1"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:3" ht="16.8" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="119" t="s">
+        <v>3452</v>
+      </c>
+      <c r="B36" s="120"/>
+      <c r="C36" s="69" t="s">
+        <v>3451</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A36:B36"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please select either &quot;Standard&quot; or &quot;Holiday&quot; from the provided drop down menu. " sqref="C12" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please select either &quot;Standard&quot; or &quot;Holiday&quot; from the provided drop down menu. " sqref="C12 C36" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Standard, Holiday"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17249,7 +18226,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:D18">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="87" priority="1">
       <formula>AND($A2=$G$2,A$1=$G$3)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -55777,7 +56754,7 @@
   <sheetPr>
     <tabColor theme="9" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:R35"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
@@ -55788,7 +56765,7 @@
     <col min="7" max="7" width="16.44140625" style="98" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>136</v>
       </c>
@@ -55810,8 +56787,14 @@
       <c r="G1" s="1" t="s">
         <v>3518</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>3570</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3571</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="111">
         <v>41640</v>
       </c>
@@ -55835,8 +56818,16 @@
         <f t="shared" ref="G2:G25" si="0">E2/B2</f>
         <v>0.41492265696087355</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H2">
+        <f>IF(G2&lt;40%,1,0)</f>
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <f>IF(F2="Kids",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="111">
         <v>41671</v>
       </c>
@@ -55860,8 +56851,16 @@
         <f t="shared" si="0"/>
         <v>0.17524916943521596</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <f t="shared" ref="H3:H25" si="2">IF(G3&lt;40%,1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I25" si="3">IF(F3="Kids",1,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="111">
         <v>41699</v>
       </c>
@@ -55876,7 +56875,7 @@
         <v>964</v>
       </c>
       <c r="E4" s="8">
-        <f t="shared" ref="E4:E19" si="2">B4-D4</f>
+        <f t="shared" ref="E4:E19" si="4">B4-D4</f>
         <v>980</v>
       </c>
       <c r="F4" s="2" t="s">
@@ -55886,8 +56885,16 @@
         <f t="shared" si="0"/>
         <v>0.50411522633744854</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="111">
         <v>41730</v>
       </c>
@@ -55902,7 +56909,7 @@
         <v>830</v>
       </c>
       <c r="E5" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>913</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -55912,8 +56919,16 @@
         <f t="shared" si="0"/>
         <v>0.52380952380952384</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="111">
         <v>41760</v>
       </c>
@@ -55928,7 +56943,7 @@
         <v>910</v>
       </c>
       <c r="E6" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>699</v>
       </c>
       <c r="F6" s="2" t="s">
@@ -55938,8 +56953,16 @@
         <f t="shared" si="0"/>
         <v>0.43443132380360472</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="111">
         <v>41791</v>
       </c>
@@ -55954,7 +56977,7 @@
         <v>909</v>
       </c>
       <c r="E7" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>585</v>
       </c>
       <c r="F7" s="2" t="s">
@@ -55964,8 +56987,16 @@
         <f t="shared" si="0"/>
         <v>0.39156626506024095</v>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="111">
         <v>41821</v>
       </c>
@@ -55980,7 +57011,7 @@
         <v>830</v>
       </c>
       <c r="E8" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1129</v>
       </c>
       <c r="F8" s="2" t="s">
@@ -55990,8 +57021,16 @@
         <f t="shared" si="0"/>
         <v>0.57631444614599281</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="111">
         <v>41852</v>
       </c>
@@ -56006,7 +57045,7 @@
         <v>906</v>
       </c>
       <c r="E9" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>962</v>
       </c>
       <c r="F9" s="2" t="s">
@@ -56016,8 +57055,16 @@
         <f t="shared" si="0"/>
         <v>0.51498929336188437</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="111">
         <v>41883</v>
       </c>
@@ -56032,7 +57079,7 @@
         <v>606</v>
       </c>
       <c r="E10" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>556</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -56042,8 +57089,16 @@
         <f t="shared" si="0"/>
         <v>0.47848537005163511</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="111">
         <v>41913</v>
       </c>
@@ -56058,7 +57113,7 @@
         <v>943</v>
       </c>
       <c r="E11" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>481</v>
       </c>
       <c r="F11" s="2" t="s">
@@ -56068,8 +57123,16 @@
         <f t="shared" si="0"/>
         <v>0.3377808988764045</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="111">
         <v>41944</v>
       </c>
@@ -56084,7 +57147,7 @@
         <v>801</v>
       </c>
       <c r="E12" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>431</v>
       </c>
       <c r="F12" s="2" t="s">
@@ -56094,8 +57157,16 @@
         <f t="shared" si="0"/>
         <v>0.34983766233766234</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="111">
         <v>41974</v>
       </c>
@@ -56110,7 +57181,7 @@
         <v>786</v>
       </c>
       <c r="E13" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>952</v>
       </c>
       <c r="F13" s="2" t="s">
@@ -56120,8 +57191,16 @@
         <f t="shared" si="0"/>
         <v>0.54775604142692746</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="111">
         <v>42005</v>
       </c>
@@ -56136,7 +57215,7 @@
         <v>575</v>
       </c>
       <c r="E14" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>860</v>
       </c>
       <c r="F14" s="2" t="s">
@@ -56146,8 +57225,16 @@
         <f t="shared" si="0"/>
         <v>0.5993031358885017</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H14">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="111">
         <v>42036</v>
       </c>
@@ -56162,7 +57249,7 @@
         <v>754</v>
       </c>
       <c r="E15" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1111</v>
       </c>
       <c r="F15" s="2" t="s">
@@ -56172,11 +57259,16 @@
         <f t="shared" si="0"/>
         <v>0.59571045576407511</v>
       </c>
-      <c r="R15" t="s">
-        <v>3552</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H15">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="111">
         <v>42064</v>
       </c>
@@ -56191,7 +57283,7 @@
         <v>599</v>
       </c>
       <c r="E16" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>635</v>
       </c>
       <c r="F16" s="2" t="s">
@@ -56201,8 +57293,16 @@
         <f t="shared" si="0"/>
         <v>0.51458670988654787</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="111">
         <v>42095</v>
       </c>
@@ -56217,7 +57317,7 @@
         <v>940</v>
       </c>
       <c r="E17" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>637</v>
       </c>
       <c r="F17" s="2" t="s">
@@ -56227,11 +57327,16 @@
         <f t="shared" si="0"/>
         <v>0.40393151553582751</v>
       </c>
-      <c r="R17" t="s">
-        <v>3552</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H17">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="111">
         <v>42125</v>
       </c>
@@ -56246,7 +57351,7 @@
         <v>954</v>
       </c>
       <c r="E18" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1029</v>
       </c>
       <c r="F18" s="2" t="s">
@@ -56256,8 +57361,16 @@
         <f t="shared" si="0"/>
         <v>0.51891074130105896</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H18">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="111">
         <v>42156</v>
       </c>
@@ -56272,7 +57385,7 @@
         <v>577</v>
       </c>
       <c r="E19" s="8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>779</v>
       </c>
       <c r="F19" s="2" t="s">
@@ -56282,8 +57395,16 @@
         <f t="shared" si="0"/>
         <v>0.57448377581120946</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="111">
         <v>42186</v>
       </c>
@@ -56307,8 +57428,16 @@
         <f t="shared" si="0"/>
         <v>0.47118463180362863</v>
       </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H20">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="111">
         <v>42217</v>
       </c>
@@ -56333,8 +57462,16 @@
         <f t="shared" si="0"/>
         <v>0.60243407707910746</v>
       </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="111">
         <v>42248</v>
       </c>
@@ -56358,8 +57495,16 @@
         <f t="shared" si="0"/>
         <v>0.36644364384971695</v>
       </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H22">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="111">
         <v>42278</v>
       </c>
@@ -56384,8 +57529,16 @@
         <f t="shared" si="0"/>
         <v>0.54501385041551242</v>
       </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="111">
         <v>42309</v>
       </c>
@@ -56410,8 +57563,16 @@
         <f t="shared" si="0"/>
         <v>0.4105827193569993</v>
       </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="H24">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="111">
         <v>42339</v>
       </c>
@@ -56436,96 +57597,74 @@
         <f t="shared" si="0"/>
         <v>0.66628308400460301</v>
       </c>
-      <c r="O25" t="b">
-        <f>AND(G2&lt;40%)</f>
+      <c r="H25">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O26" t="b">
-        <f t="shared" ref="O26:O35" si="3">AND(G3&lt;40%)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O27" t="b">
+      <c r="I25">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O28" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O29" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O30" t="b">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O31" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="O32" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O33" t="b">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O34" t="b">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="15:15" x14ac:dyDescent="0.3">
-      <c r="O35" t="b">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C25">
-    <cfRule type="iconSet" priority="1">
+    <cfRule type="iconSet" priority="9">
       <iconSet iconSet="3Arrows">
         <cfvo type="percent" val="0"/>
         <cfvo type="num" val="200"/>
         <cfvo type="num" val="200"/>
       </iconSet>
     </cfRule>
+    <cfRule type="expression" dxfId="24" priority="5">
+      <formula>IF(F2="Kids",1,0)</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G25">
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="10" operator="lessThan">
       <formula>0.421</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="11" operator="lessThan">
       <formula>0.421</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="12" operator="greaterThan">
       <formula>0.421</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="16" priority="13" operator="greaterThan">
       <formula>0.421</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="14" operator="lessThan">
       <formula>0.421</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>"IF(F2=""Kids"",1,0)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A25">
+    <cfRule type="expression" dxfId="23" priority="8">
+      <formula>IF(G2&lt;40%,1,0)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="7">
+      <formula>IF(F2="Kids",1,0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B25">
+    <cfRule type="expression" dxfId="21" priority="6">
+      <formula>IF(F2="Kids",1,0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D25">
+    <cfRule type="expression" dxfId="20" priority="4">
+      <formula>IF(F2="Kids",1,0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E25">
+    <cfRule type="expression" dxfId="19" priority="3">
+      <formula>IF(F2="Kids",1,0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F25">
+    <cfRule type="expression" dxfId="18" priority="2">
+      <formula>IF(F2="Kids",1,0)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -56559,7 +57698,7 @@
       </c>
       <c r="C2" s="113">
         <f ca="1">TODAY()</f>
-        <v>46228</v>
+        <v>46230</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -56568,7 +57707,7 @@
       </c>
       <c r="C3" s="114">
         <f ca="1">NOW()</f>
-        <v>46228.381456944444</v>
+        <v>46230.760147106485</v>
       </c>
       <c r="E3" s="109" t="s">
         <v>3544</v>
@@ -56594,7 +57733,7 @@
       </c>
       <c r="F5" s="108">
         <f ca="1">_xlfn.DAYS(F3,C2)</f>
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -56616,7 +57755,7 @@
       </c>
       <c r="C7" s="106">
         <f ca="1">DAY(TODAY())</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>3538</v>
@@ -56630,7 +57769,7 @@
       </c>
       <c r="C8" s="106">
         <f ca="1">HOUR(NOW())</f>
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -56639,7 +57778,7 @@
       </c>
       <c r="C9" s="106">
         <f ca="1">MINUTE(NOW())</f>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>3535</v>
@@ -56652,7 +57791,7 @@
       </c>
       <c r="C10" s="105">
         <f ca="1">SECOND(NOW())</f>
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="E10" s="9" t="s">
         <v>3533</v>
@@ -57693,7 +58832,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="131" t="s">
-        <v>3553</v>
+        <v>3552</v>
       </c>
       <c r="B1" s="131"/>
       <c r="C1" s="131"/>
@@ -57961,7 +59100,10 @@
       <c r="G6" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="H6" s="47"/>
+      <c r="H6" s="47" cm="1">
+        <f t="array" ref="H6">SUM(IF(E2:E16&gt;D2:D16,1,0))</f>
+        <v>9</v>
+      </c>
       <c r="I6" s="12"/>
       <c r="J6" s="39"/>
     </row>
@@ -58225,7 +59367,7 @@
         <v>2150</v>
       </c>
       <c r="K5" s="49" t="s">
-        <v>3555</v>
+        <v>3554</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -58407,7 +59549,7 @@
         <v>11300</v>
       </c>
       <c r="K12" s="49" t="s">
-        <v>3556</v>
+        <v>3555</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -58533,7 +59675,7 @@
         <v>37250</v>
       </c>
       <c r="K17" s="49" t="s">
-        <v>3557</v>
+        <v>3556</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>